<commit_message>
Excel de la tarea: individual
</commit_message>
<xml_diff>
--- a/material/Tarea-S1-Estado-Financiero.xlsx
+++ b/material/Tarea-S1-Estado-Financiero.xlsx
@@ -567,7 +567,7 @@
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Tarea en grupo · Sesión 1 · AI Productivity Engineering (eIA)</t>
+          <t>Tarea individual · Sesión 1 · AI Productivity Engineering (eIA)</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Grupos de 3 a 4 personas. Entrega antes de la próxima sesión.</t>
+          <t>Tarea individual. Entrega en https://unimauro.github.io/curso-ia-productividad/entregar.html hasta el jueves 1 de octubre, 6:59 p. m. (hora de Lima).</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Conclusión del grupo (3 a 5 líneas):</t>
+          <t>Tu conclusión (3 a 5 líneas):</t>
         </is>
       </c>
       <c r="B14" s="1" t="n"/>

</xml_diff>